<commit_message>
Beispieldaten durch simulierte Daten ersetzen
BspDaten wird mit data-raw/BspDaten.R reproduzierbar erzeugt (gleicher Aufbau, erfundene Fachbereiche, Lorem ipsum). Beispiel-Berichtstabelle: Sonderauswertung statt Studienberatung. Vergleichsausgaben der Tests neu erzeugt.
</commit_message>
<xml_diff>
--- a/inst/extdata/beispiel_berichte.xlsx
+++ b/inst/extdata/beispiel_berichte.xlsx
@@ -519,7 +519,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Studienberatung</t>
+          <t>Sonderauswertung</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Befragung 2024: Studienberatung</t>
+          <t>Befragung 2024: Sonderauswertung</t>
         </is>
       </c>
     </row>

</xml_diff>